<commit_message>
Remove benchmark percentile columns and update call grading data
</commit_message>
<xml_diff>
--- a/MAS_Call_Grading_Raw_Data.xlsx
+++ b/MAS_Call_Grading_Raw_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF14A11E-555C-42F6-8CE0-F8DEADAEFFCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76F2FF37-1921-4B37-A7F2-210530B048F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="130" yWindow="150" windowWidth="31410" windowHeight="13490" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
+    <workbookView xWindow="5680" yWindow="350" windowWidth="21240" windowHeight="13490" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="58">
   <si>
     <t>AssociateName</t>
   </si>
@@ -208,6 +208,9 @@
   </si>
   <si>
     <t>Thomas.Gordon@lplfinancial.com</t>
+  </si>
+  <si>
+    <t>April</t>
   </si>
 </sst>
 </file>
@@ -259,7 +262,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -274,8 +277,14 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -322,8 +331,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O8" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:O8" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O17" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:O17" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{F3FB1979-6840-4EDA-8F75-C44587A3E01A}" name="AssociateName"/>
     <tableColumn id="2" xr3:uid="{13759531-2D3E-4AB5-99AA-3CEAD45C9112}" name="ManagerTeam"/>
@@ -676,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E2710C-161E-4D4C-A0A9-FF139CE211A3}">
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.54296875" customWidth="1"/>
@@ -968,7 +977,7 @@
       <c r="L6" s="1">
         <v>90</v>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="2">
         <v>0.9</v>
       </c>
       <c r="N6" s="1" t="s">
@@ -1015,7 +1024,7 @@
       <c r="L7" s="1">
         <v>100</v>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="2">
         <v>1</v>
       </c>
       <c r="N7" s="1" t="s">
@@ -1062,13 +1071,436 @@
       <c r="L8" s="1">
         <v>100</v>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="2">
         <v>1</v>
       </c>
       <c r="N8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="O8" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="5">
+        <v>46104</v>
+      </c>
+      <c r="D9" s="1">
+        <v>5</v>
+      </c>
+      <c r="E9" s="1">
+        <v>20</v>
+      </c>
+      <c r="F9" s="1">
+        <v>30</v>
+      </c>
+      <c r="G9" s="1">
+        <v>20</v>
+      </c>
+      <c r="H9" s="1">
+        <v>20</v>
+      </c>
+      <c r="I9" s="1">
+        <v>5</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L9" s="1">
+        <v>100</v>
+      </c>
+      <c r="M9" s="2">
+        <v>1</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O9" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="5">
+        <v>46119</v>
+      </c>
+      <c r="D10" s="1">
+        <v>5</v>
+      </c>
+      <c r="E10" s="1">
+        <v>20</v>
+      </c>
+      <c r="F10" s="1">
+        <v>30</v>
+      </c>
+      <c r="G10" s="1">
+        <v>20</v>
+      </c>
+      <c r="H10" s="1">
+        <v>15</v>
+      </c>
+      <c r="I10" s="1">
+        <v>5</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L10" s="1">
+        <v>95</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="O10" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="5">
+        <v>46114</v>
+      </c>
+      <c r="D11" s="1">
+        <v>5</v>
+      </c>
+      <c r="E11" s="1">
+        <v>20</v>
+      </c>
+      <c r="F11" s="1">
+        <v>20</v>
+      </c>
+      <c r="G11" s="1">
+        <v>20</v>
+      </c>
+      <c r="H11" s="1">
+        <v>10</v>
+      </c>
+      <c r="I11" s="1">
+        <v>5</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L11" s="1">
+        <v>80</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="O11" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="5">
+        <v>46101</v>
+      </c>
+      <c r="D12" s="1">
+        <v>5</v>
+      </c>
+      <c r="E12" s="1">
+        <v>20</v>
+      </c>
+      <c r="F12" s="1">
+        <v>30</v>
+      </c>
+      <c r="G12" s="1">
+        <v>20</v>
+      </c>
+      <c r="H12" s="1">
+        <v>20</v>
+      </c>
+      <c r="I12" s="1">
+        <v>5</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L12" s="1">
+        <v>100</v>
+      </c>
+      <c r="M12" s="2">
+        <v>1</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O12" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="5">
+        <v>46100</v>
+      </c>
+      <c r="D13" s="1">
+        <v>5</v>
+      </c>
+      <c r="E13" s="1">
+        <v>20</v>
+      </c>
+      <c r="F13" s="1">
+        <v>30</v>
+      </c>
+      <c r="G13" s="1">
+        <v>20</v>
+      </c>
+      <c r="H13" s="1">
+        <v>20</v>
+      </c>
+      <c r="I13" s="1">
+        <v>5</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L13" s="1">
+        <v>100</v>
+      </c>
+      <c r="M13" s="2">
+        <v>1</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O13" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="5">
+        <v>46094</v>
+      </c>
+      <c r="D14" s="1">
+        <v>5</v>
+      </c>
+      <c r="E14" s="1">
+        <v>20</v>
+      </c>
+      <c r="F14" s="1">
+        <v>30</v>
+      </c>
+      <c r="G14" s="1">
+        <v>20</v>
+      </c>
+      <c r="H14" s="1">
+        <v>15</v>
+      </c>
+      <c r="I14" s="1">
+        <v>5</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L14" s="1">
+        <v>95</v>
+      </c>
+      <c r="M14" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O14" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="5">
+        <v>46094</v>
+      </c>
+      <c r="D15" s="1">
+        <v>5</v>
+      </c>
+      <c r="E15" s="1">
+        <v>20</v>
+      </c>
+      <c r="F15" s="1">
+        <v>30</v>
+      </c>
+      <c r="G15" s="1">
+        <v>20</v>
+      </c>
+      <c r="H15" s="1">
+        <v>20</v>
+      </c>
+      <c r="I15" s="1">
+        <v>5</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L15" s="1">
+        <v>100</v>
+      </c>
+      <c r="M15" s="2">
+        <v>1</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O15" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="5">
+        <v>46101</v>
+      </c>
+      <c r="D16" s="1">
+        <v>5</v>
+      </c>
+      <c r="E16" s="1">
+        <v>20</v>
+      </c>
+      <c r="F16" s="1">
+        <v>30</v>
+      </c>
+      <c r="G16" s="1">
+        <v>20</v>
+      </c>
+      <c r="H16" s="1">
+        <v>20</v>
+      </c>
+      <c r="I16" s="1">
+        <v>5</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L16" s="1">
+        <v>100</v>
+      </c>
+      <c r="M16" s="2">
+        <v>1</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O16" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="7">
+        <v>46113</v>
+      </c>
+      <c r="D17" s="6">
+        <v>5</v>
+      </c>
+      <c r="E17" s="6">
+        <v>20</v>
+      </c>
+      <c r="F17" s="6">
+        <v>30</v>
+      </c>
+      <c r="G17" s="6">
+        <v>20</v>
+      </c>
+      <c r="H17" s="6">
+        <v>0</v>
+      </c>
+      <c r="I17" s="6">
+        <v>5</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L17" s="6">
+        <v>0</v>
+      </c>
+      <c r="M17" s="8">
+        <v>0</v>
+      </c>
+      <c r="N17" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="O17" s="6">
         <v>2026</v>
       </c>
     </row>
@@ -1374,6 +1806,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
+    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B7CF5D77C2318A48AE3D01AED053E969" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7f98047a509e9e082d0d58dfbe71352c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c3d3890c-cedb-4996-8d69-32a58562dce0" xmlns:ns3="081083fe-e475-436e-8ac6-57ab24d1081c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="361f48e45990901628f9319c45e78890" ns2:_="" ns3:_="">
     <xsd:import namespace="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
@@ -1624,29 +2078,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
-    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AAD6C53-AA8B-4861-BD9E-3003633B2469}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E95F4425-7749-4603-B4BA-980799E13416}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1663,29 +2120,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AAD6C53-AA8B-4861-BD9E-3003633B2469}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update MAS Call Grading Raw Data 0413
</commit_message>
<xml_diff>
--- a/MAS_Call_Grading_Raw_Data.xlsx
+++ b/MAS_Call_Grading_Raw_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F56F01CB-C0D8-4268-80DE-AFE9278C4E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{802A1E98-F0A2-46EE-BF49-63C3E9C1EF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1750" yWindow="460" windowWidth="26510" windowHeight="13490" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
+    <workbookView xWindow="1110" yWindow="140" windowWidth="22240" windowHeight="13490" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="58">
   <si>
     <t>AssociateName</t>
   </si>
@@ -126,6 +126,12 @@
     <t>April</t>
   </si>
   <si>
+    <t>Marnia Vance</t>
+  </si>
+  <si>
+    <t>Michael Chen</t>
+  </si>
+  <si>
     <t>ManagerName</t>
   </si>
   <si>
@@ -165,13 +171,7 @@
     <t>Tyler.Rainford@lplfinancial.com</t>
   </si>
   <si>
-    <t>Marnia Vance</t>
-  </si>
-  <si>
     <t>Marnia.Vance@lplfinancial.com</t>
-  </si>
-  <si>
-    <t>Michael Chen</t>
   </si>
   <si>
     <t>Michael.Chen@lplfinancial.com</t>
@@ -325,8 +325,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O20" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:O20" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O28" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:O28" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{F3FB1979-6840-4EDA-8F75-C44587A3E01A}" name="AssociateName"/>
     <tableColumn id="2" xr3:uid="{13759531-2D3E-4AB5-99AA-3CEAD45C9112}" name="ManagerTeam"/>
@@ -679,7 +679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E2710C-161E-4D4C-A0A9-FF139CE211A3}">
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.54296875" customWidth="1"/>
@@ -1488,7 +1488,7 @@
       <c r="L17" s="1">
         <v>85</v>
       </c>
-      <c r="M17" s="6">
+      <c r="M17" s="2">
         <v>0.85</v>
       </c>
       <c r="N17" s="1" t="s">
@@ -1500,7 +1500,7 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>16</v>
@@ -1535,7 +1535,7 @@
       <c r="L18" s="1">
         <v>85</v>
       </c>
-      <c r="M18" s="6">
+      <c r="M18" s="2">
         <v>0.85</v>
       </c>
       <c r="N18" s="1" t="s">
@@ -1547,7 +1547,7 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>16</v>
@@ -1582,7 +1582,7 @@
       <c r="L19" s="1">
         <v>90</v>
       </c>
-      <c r="M19" s="6">
+      <c r="M19" s="2">
         <v>0.9</v>
       </c>
       <c r="N19" s="1" t="s">
@@ -1629,13 +1629,389 @@
       <c r="L20" s="1">
         <v>85</v>
       </c>
-      <c r="M20" s="6">
+      <c r="M20" s="2">
         <v>0.85</v>
       </c>
       <c r="N20" s="1" t="s">
         <v>19</v>
       </c>
       <c r="O20" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="5">
+        <v>46101</v>
+      </c>
+      <c r="D21" s="1">
+        <v>5</v>
+      </c>
+      <c r="E21" s="1">
+        <v>20</v>
+      </c>
+      <c r="F21" s="1">
+        <v>30</v>
+      </c>
+      <c r="G21" s="1">
+        <v>20</v>
+      </c>
+      <c r="H21" s="1">
+        <v>20</v>
+      </c>
+      <c r="I21" s="1">
+        <v>5</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L21" s="1">
+        <v>100</v>
+      </c>
+      <c r="M21" s="6">
+        <v>1</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O21" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="5">
+        <v>46113</v>
+      </c>
+      <c r="D22" s="1">
+        <v>5</v>
+      </c>
+      <c r="E22" s="1">
+        <v>20</v>
+      </c>
+      <c r="F22" s="1">
+        <v>30</v>
+      </c>
+      <c r="G22" s="1">
+        <v>20</v>
+      </c>
+      <c r="H22" s="1">
+        <v>20</v>
+      </c>
+      <c r="I22" s="1">
+        <v>5</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L22" s="1">
+        <v>100</v>
+      </c>
+      <c r="M22" s="6">
+        <v>1</v>
+      </c>
+      <c r="N22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O22" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="5">
+        <v>46120</v>
+      </c>
+      <c r="D23" s="1">
+        <v>5</v>
+      </c>
+      <c r="E23" s="1">
+        <v>20</v>
+      </c>
+      <c r="F23" s="1">
+        <v>30</v>
+      </c>
+      <c r="G23" s="1">
+        <v>20</v>
+      </c>
+      <c r="H23" s="1">
+        <v>20</v>
+      </c>
+      <c r="I23" s="1">
+        <v>5</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L23" s="1">
+        <v>100</v>
+      </c>
+      <c r="M23" s="6">
+        <v>1</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O23" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="5">
+        <v>46121</v>
+      </c>
+      <c r="D24" s="1">
+        <v>5</v>
+      </c>
+      <c r="E24" s="1">
+        <v>20</v>
+      </c>
+      <c r="F24" s="1">
+        <v>30</v>
+      </c>
+      <c r="G24" s="1">
+        <v>20</v>
+      </c>
+      <c r="H24" s="1">
+        <v>20</v>
+      </c>
+      <c r="I24" s="1">
+        <v>5</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L24" s="1">
+        <v>100</v>
+      </c>
+      <c r="M24" s="6">
+        <v>1</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O24" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A25" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="5">
+        <v>46120</v>
+      </c>
+      <c r="D25" s="1">
+        <v>5</v>
+      </c>
+      <c r="E25" s="1">
+        <v>20</v>
+      </c>
+      <c r="F25" s="1">
+        <v>30</v>
+      </c>
+      <c r="G25" s="1">
+        <v>20</v>
+      </c>
+      <c r="H25" s="1">
+        <v>10</v>
+      </c>
+      <c r="I25" s="1">
+        <v>5</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L25" s="1">
+        <v>90</v>
+      </c>
+      <c r="M25" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O25" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="5">
+        <v>46121</v>
+      </c>
+      <c r="D26" s="1">
+        <v>5</v>
+      </c>
+      <c r="E26" s="1">
+        <v>20</v>
+      </c>
+      <c r="F26" s="1">
+        <v>30</v>
+      </c>
+      <c r="G26" s="1">
+        <v>10</v>
+      </c>
+      <c r="H26" s="1">
+        <v>0</v>
+      </c>
+      <c r="I26" s="1">
+        <v>5</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L26" s="1">
+        <v>0</v>
+      </c>
+      <c r="M26" s="6">
+        <v>0</v>
+      </c>
+      <c r="N26" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O26" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A27" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="5">
+        <v>46100</v>
+      </c>
+      <c r="D27" s="1">
+        <v>5</v>
+      </c>
+      <c r="E27" s="1">
+        <v>20</v>
+      </c>
+      <c r="F27" s="1">
+        <v>30</v>
+      </c>
+      <c r="G27" s="1">
+        <v>20</v>
+      </c>
+      <c r="H27" s="1">
+        <v>20</v>
+      </c>
+      <c r="I27" s="1">
+        <v>5</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L27" s="1">
+        <v>100</v>
+      </c>
+      <c r="M27" s="6">
+        <v>1</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O27" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="5">
+        <v>46100</v>
+      </c>
+      <c r="D28" s="1">
+        <v>5</v>
+      </c>
+      <c r="E28" s="1">
+        <v>10</v>
+      </c>
+      <c r="F28" s="1">
+        <v>15</v>
+      </c>
+      <c r="G28" s="1">
+        <v>10</v>
+      </c>
+      <c r="H28" s="1">
+        <v>10</v>
+      </c>
+      <c r="I28" s="1">
+        <v>5</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L28" s="1">
+        <v>55</v>
+      </c>
+      <c r="M28" s="6">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="N28" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O28" s="1">
         <v>2026</v>
       </c>
     </row>
@@ -1667,30 +2043,30 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -1701,30 +2077,30 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -1735,61 +2111,61 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
         <v>45</v>
@@ -1905,10 +2281,10 @@
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E15" t="s">
         <v>56</v>
@@ -2216,15 +2592,15 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>

</xml_diff>

<commit_message>
MAS Call Grading 0420
</commit_message>
<xml_diff>
--- a/MAS_Call_Grading_Raw_Data.xlsx
+++ b/MAS_Call_Grading_Raw_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{802A1E98-F0A2-46EE-BF49-63C3E9C1EF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8E0DFE8-41F6-4D59-A57B-E03ACA22F020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1110" yWindow="140" windowWidth="22240" windowHeight="13490" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
+    <workbookView xWindow="470" yWindow="0" windowWidth="22910" windowHeight="13490" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="58">
   <si>
     <t>AssociateName</t>
   </si>
@@ -132,6 +132,18 @@
     <t>Michael Chen</t>
   </si>
   <si>
+    <t>TyKee Walmsley</t>
+  </si>
+  <si>
+    <t>Tyler Rainford</t>
+  </si>
+  <si>
+    <t>Seshu Chivukula</t>
+  </si>
+  <si>
+    <t>Breanna Stringfellow</t>
+  </si>
+  <si>
     <t>ManagerName</t>
   </si>
   <si>
@@ -141,9 +153,6 @@
     <t>AssociateEmail</t>
   </si>
   <si>
-    <t>Seshu Chivukula</t>
-  </si>
-  <si>
     <t>Charles Bumgardner</t>
   </si>
   <si>
@@ -156,18 +165,12 @@
     <t>Connie.Serrano@lplfinancial.com</t>
   </si>
   <si>
-    <t>TyKee Walmsley</t>
-  </si>
-  <si>
     <t>TyKee.Walmsley@lplfinancial.com</t>
   </si>
   <si>
     <t>Kelly.Acevedo@lplfinancial.com</t>
   </si>
   <si>
-    <t>Tyler Rainford</t>
-  </si>
-  <si>
     <t>Tyler.Rainford@lplfinancial.com</t>
   </si>
   <si>
@@ -202,9 +205,6 @@
   </si>
   <si>
     <t>Marcus.McDowell@lplfinancial.com</t>
-  </si>
-  <si>
-    <t>Breanna Stringfellow</t>
   </si>
   <si>
     <t>Breanna.Stringfellow@lplfinancial.com</t>
@@ -325,8 +325,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O28" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:O28" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O37" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:O37" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{F3FB1979-6840-4EDA-8F75-C44587A3E01A}" name="AssociateName"/>
     <tableColumn id="2" xr3:uid="{13759531-2D3E-4AB5-99AA-3CEAD45C9112}" name="ManagerTeam"/>
@@ -679,7 +679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E2710C-161E-4D4C-A0A9-FF139CE211A3}">
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.54296875" customWidth="1"/>
@@ -1676,7 +1676,7 @@
       <c r="L21" s="1">
         <v>100</v>
       </c>
-      <c r="M21" s="6">
+      <c r="M21" s="2">
         <v>1</v>
       </c>
       <c r="N21" s="1" t="s">
@@ -1688,7 +1688,7 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>16</v>
@@ -1723,7 +1723,7 @@
       <c r="L22" s="1">
         <v>100</v>
       </c>
-      <c r="M22" s="6">
+      <c r="M22" s="2">
         <v>1</v>
       </c>
       <c r="N22" s="1" t="s">
@@ -1735,7 +1735,7 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>16</v>
@@ -1770,7 +1770,7 @@
       <c r="L23" s="1">
         <v>100</v>
       </c>
-      <c r="M23" s="6">
+      <c r="M23" s="2">
         <v>1</v>
       </c>
       <c r="N23" s="1" t="s">
@@ -1782,7 +1782,7 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>16</v>
@@ -1817,7 +1817,7 @@
       <c r="L24" s="1">
         <v>100</v>
       </c>
-      <c r="M24" s="6">
+      <c r="M24" s="2">
         <v>1</v>
       </c>
       <c r="N24" s="1" t="s">
@@ -1829,7 +1829,7 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>16</v>
@@ -1864,7 +1864,7 @@
       <c r="L25" s="1">
         <v>90</v>
       </c>
-      <c r="M25" s="6">
+      <c r="M25" s="2">
         <v>0.9</v>
       </c>
       <c r="N25" s="1" t="s">
@@ -1911,7 +1911,7 @@
       <c r="L26" s="1">
         <v>0</v>
       </c>
-      <c r="M26" s="6">
+      <c r="M26" s="2">
         <v>0</v>
       </c>
       <c r="N26" s="1" t="s">
@@ -1958,7 +1958,7 @@
       <c r="L27" s="1">
         <v>100</v>
       </c>
-      <c r="M27" s="6">
+      <c r="M27" s="2">
         <v>1</v>
       </c>
       <c r="N27" s="1" t="s">
@@ -2005,13 +2005,436 @@
       <c r="L28" s="1">
         <v>55</v>
       </c>
-      <c r="M28" s="6">
+      <c r="M28" s="2">
         <v>0.55000000000000004</v>
       </c>
       <c r="N28" s="1" t="s">
         <v>19</v>
       </c>
       <c r="O28" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="5">
+        <v>46106</v>
+      </c>
+      <c r="D29" s="1">
+        <v>5</v>
+      </c>
+      <c r="E29" s="1">
+        <v>20</v>
+      </c>
+      <c r="F29" s="1">
+        <v>30</v>
+      </c>
+      <c r="G29" s="1">
+        <v>20</v>
+      </c>
+      <c r="H29" s="1">
+        <v>20</v>
+      </c>
+      <c r="I29" s="1">
+        <v>5</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L29" s="1">
+        <v>100</v>
+      </c>
+      <c r="M29" s="6">
+        <v>1</v>
+      </c>
+      <c r="N29" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O29" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="5">
+        <v>46106</v>
+      </c>
+      <c r="D30" s="1">
+        <v>5</v>
+      </c>
+      <c r="E30" s="1">
+        <v>20</v>
+      </c>
+      <c r="F30" s="1">
+        <v>30</v>
+      </c>
+      <c r="G30" s="1">
+        <v>20</v>
+      </c>
+      <c r="H30" s="1">
+        <v>20</v>
+      </c>
+      <c r="I30" s="1">
+        <v>5</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L30" s="1">
+        <v>100</v>
+      </c>
+      <c r="M30" s="6">
+        <v>1</v>
+      </c>
+      <c r="N30" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O30" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A31" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="5">
+        <v>46127</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0</v>
+      </c>
+      <c r="E31" s="1">
+        <v>20</v>
+      </c>
+      <c r="F31" s="1">
+        <v>30</v>
+      </c>
+      <c r="G31" s="1">
+        <v>20</v>
+      </c>
+      <c r="H31" s="1">
+        <v>20</v>
+      </c>
+      <c r="I31" s="1">
+        <v>0</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L31" s="1">
+        <v>0</v>
+      </c>
+      <c r="M31" s="6">
+        <v>0</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O31" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A32" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="5">
+        <v>46128</v>
+      </c>
+      <c r="D32" s="1">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1">
+        <v>20</v>
+      </c>
+      <c r="F32" s="1">
+        <v>30</v>
+      </c>
+      <c r="G32" s="1">
+        <v>20</v>
+      </c>
+      <c r="H32" s="1">
+        <v>20</v>
+      </c>
+      <c r="I32" s="1">
+        <v>5</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L32" s="1">
+        <v>0</v>
+      </c>
+      <c r="M32" s="6">
+        <v>0</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O32" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A33" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="5">
+        <v>46127</v>
+      </c>
+      <c r="D33" s="1">
+        <v>5</v>
+      </c>
+      <c r="E33" s="1">
+        <v>20</v>
+      </c>
+      <c r="F33" s="1">
+        <v>30</v>
+      </c>
+      <c r="G33" s="1">
+        <v>20</v>
+      </c>
+      <c r="H33" s="1">
+        <v>20</v>
+      </c>
+      <c r="I33" s="1">
+        <v>5</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L33" s="1">
+        <v>100</v>
+      </c>
+      <c r="M33" s="6">
+        <v>1</v>
+      </c>
+      <c r="N33" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O33" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="5">
+        <v>46127</v>
+      </c>
+      <c r="D34" s="1">
+        <v>5</v>
+      </c>
+      <c r="E34" s="1">
+        <v>20</v>
+      </c>
+      <c r="F34" s="1">
+        <v>30</v>
+      </c>
+      <c r="G34" s="1">
+        <v>20</v>
+      </c>
+      <c r="H34" s="1">
+        <v>20</v>
+      </c>
+      <c r="I34" s="1">
+        <v>5</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L34" s="1">
+        <v>100</v>
+      </c>
+      <c r="M34" s="6">
+        <v>1</v>
+      </c>
+      <c r="N34" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O34" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="5">
+        <v>46128</v>
+      </c>
+      <c r="D35" s="1">
+        <v>5</v>
+      </c>
+      <c r="E35" s="1">
+        <v>20</v>
+      </c>
+      <c r="F35" s="1">
+        <v>30</v>
+      </c>
+      <c r="G35" s="1">
+        <v>20</v>
+      </c>
+      <c r="H35" s="1">
+        <v>20</v>
+      </c>
+      <c r="I35" s="1">
+        <v>5</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K35" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L35" s="1">
+        <v>100</v>
+      </c>
+      <c r="M35" s="6">
+        <v>1</v>
+      </c>
+      <c r="N35" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O35" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C36" s="5">
+        <v>46127</v>
+      </c>
+      <c r="D36" s="1">
+        <v>5</v>
+      </c>
+      <c r="E36" s="1">
+        <v>20</v>
+      </c>
+      <c r="F36" s="1">
+        <v>30</v>
+      </c>
+      <c r="G36" s="1">
+        <v>20</v>
+      </c>
+      <c r="H36" s="1">
+        <v>20</v>
+      </c>
+      <c r="I36" s="1">
+        <v>5</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K36" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L36" s="1">
+        <v>100</v>
+      </c>
+      <c r="M36" s="6">
+        <v>1</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O36" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C37" s="5">
+        <v>46128</v>
+      </c>
+      <c r="D37" s="1">
+        <v>5</v>
+      </c>
+      <c r="E37" s="1">
+        <v>20</v>
+      </c>
+      <c r="F37" s="1">
+        <v>30</v>
+      </c>
+      <c r="G37" s="1">
+        <v>20</v>
+      </c>
+      <c r="H37" s="1">
+        <v>0</v>
+      </c>
+      <c r="I37" s="1">
+        <v>5</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K37" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L37" s="1">
+        <v>0</v>
+      </c>
+      <c r="M37" s="6">
+        <v>0</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O37" s="1">
         <v>2026</v>
       </c>
     </row>
@@ -2043,30 +2466,30 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2077,30 +2500,30 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -2111,30 +2534,30 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -2145,13 +2568,13 @@
         <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -2162,13 +2585,13 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -2179,30 +2602,30 @@
         <v>21</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
         <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -2213,13 +2636,13 @@
         <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -2230,13 +2653,13 @@
         <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -2247,13 +2670,13 @@
         <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -2264,27 +2687,27 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
         <v>16</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
         <v>56</v>
@@ -2298,10 +2721,10 @@
         <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E16" t="s">
         <v>57</v>
@@ -2592,16 +3015,16 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update charts, benchmark labels, and call grading data
</commit_message>
<xml_diff>
--- a/MAS_Call_Grading_Raw_Data.xlsx
+++ b/MAS_Call_Grading_Raw_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8E0DFE8-41F6-4D59-A57B-E03ACA22F020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DE82187-698C-4490-B793-932701D9FE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="470" yWindow="0" windowWidth="22910" windowHeight="13490" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
+    <workbookView xWindow="-60" yWindow="460" windowWidth="28450" windowHeight="12670" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="58">
   <si>
     <t>AssociateName</t>
   </si>
@@ -325,8 +325,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O37" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:O37" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O52" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:O52" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{F3FB1979-6840-4EDA-8F75-C44587A3E01A}" name="AssociateName"/>
     <tableColumn id="2" xr3:uid="{13759531-2D3E-4AB5-99AA-3CEAD45C9112}" name="ManagerTeam"/>
@@ -679,7 +679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E2710C-161E-4D4C-A0A9-FF139CE211A3}">
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.54296875" customWidth="1"/>
@@ -2052,7 +2052,7 @@
       <c r="L29" s="1">
         <v>100</v>
       </c>
-      <c r="M29" s="6">
+      <c r="M29" s="2">
         <v>1</v>
       </c>
       <c r="N29" s="1" t="s">
@@ -2099,7 +2099,7 @@
       <c r="L30" s="1">
         <v>100</v>
       </c>
-      <c r="M30" s="6">
+      <c r="M30" s="2">
         <v>1</v>
       </c>
       <c r="N30" s="1" t="s">
@@ -2146,7 +2146,7 @@
       <c r="L31" s="1">
         <v>0</v>
       </c>
-      <c r="M31" s="6">
+      <c r="M31" s="2">
         <v>0</v>
       </c>
       <c r="N31" s="1" t="s">
@@ -2193,7 +2193,7 @@
       <c r="L32" s="1">
         <v>0</v>
       </c>
-      <c r="M32" s="6">
+      <c r="M32" s="2">
         <v>0</v>
       </c>
       <c r="N32" s="1" t="s">
@@ -2240,7 +2240,7 @@
       <c r="L33" s="1">
         <v>100</v>
       </c>
-      <c r="M33" s="6">
+      <c r="M33" s="2">
         <v>1</v>
       </c>
       <c r="N33" s="1" t="s">
@@ -2287,7 +2287,7 @@
       <c r="L34" s="1">
         <v>100</v>
       </c>
-      <c r="M34" s="6">
+      <c r="M34" s="2">
         <v>1</v>
       </c>
       <c r="N34" s="1" t="s">
@@ -2334,7 +2334,7 @@
       <c r="L35" s="1">
         <v>100</v>
       </c>
-      <c r="M35" s="6">
+      <c r="M35" s="2">
         <v>1</v>
       </c>
       <c r="N35" s="1" t="s">
@@ -2381,7 +2381,7 @@
       <c r="L36" s="1">
         <v>100</v>
       </c>
-      <c r="M36" s="6">
+      <c r="M36" s="2">
         <v>1</v>
       </c>
       <c r="N36" s="1" t="s">
@@ -2428,13 +2428,718 @@
       <c r="L37" s="1">
         <v>0</v>
       </c>
-      <c r="M37" s="6">
+      <c r="M37" s="2">
         <v>0</v>
       </c>
       <c r="N37" s="1" t="s">
         <v>28</v>
       </c>
       <c r="O37" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" s="5">
+        <v>46125</v>
+      </c>
+      <c r="D38" s="1">
+        <v>5</v>
+      </c>
+      <c r="E38" s="1">
+        <v>5</v>
+      </c>
+      <c r="F38" s="1">
+        <v>25</v>
+      </c>
+      <c r="G38" s="1">
+        <v>20</v>
+      </c>
+      <c r="H38" s="1">
+        <v>0</v>
+      </c>
+      <c r="I38" s="1">
+        <v>5</v>
+      </c>
+      <c r="J38" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L38" s="1">
+        <v>0</v>
+      </c>
+      <c r="M38" s="2">
+        <v>0</v>
+      </c>
+      <c r="N38" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O38" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A39" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="5">
+        <v>46128</v>
+      </c>
+      <c r="D39" s="1">
+        <v>5</v>
+      </c>
+      <c r="E39" s="1">
+        <v>20</v>
+      </c>
+      <c r="F39" s="1">
+        <v>25</v>
+      </c>
+      <c r="G39" s="1">
+        <v>20</v>
+      </c>
+      <c r="H39" s="1">
+        <v>0</v>
+      </c>
+      <c r="I39" s="1">
+        <v>5</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L39" s="1">
+        <v>0</v>
+      </c>
+      <c r="M39" s="2">
+        <v>0</v>
+      </c>
+      <c r="N39" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O39" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A40" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" s="5">
+        <v>46104</v>
+      </c>
+      <c r="D40" s="1">
+        <v>0</v>
+      </c>
+      <c r="E40" s="1">
+        <v>20</v>
+      </c>
+      <c r="F40" s="1">
+        <v>30</v>
+      </c>
+      <c r="G40" s="1">
+        <v>20</v>
+      </c>
+      <c r="H40" s="1">
+        <v>20</v>
+      </c>
+      <c r="I40" s="1">
+        <v>5</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L40" s="1">
+        <v>0</v>
+      </c>
+      <c r="M40" s="2">
+        <v>0</v>
+      </c>
+      <c r="N40" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O40" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A41" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" s="5">
+        <v>46112</v>
+      </c>
+      <c r="D41" s="1">
+        <v>0</v>
+      </c>
+      <c r="E41" s="1">
+        <v>10</v>
+      </c>
+      <c r="F41" s="1">
+        <v>30</v>
+      </c>
+      <c r="G41" s="1">
+        <v>20</v>
+      </c>
+      <c r="H41" s="1">
+        <v>20</v>
+      </c>
+      <c r="I41" s="1">
+        <v>0</v>
+      </c>
+      <c r="J41" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="L41" s="1">
+        <v>0</v>
+      </c>
+      <c r="M41" s="2">
+        <v>0</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O41" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A42" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" s="5">
+        <v>46111</v>
+      </c>
+      <c r="D42" s="1">
+        <v>5</v>
+      </c>
+      <c r="E42" s="1">
+        <v>20</v>
+      </c>
+      <c r="F42" s="1">
+        <v>30</v>
+      </c>
+      <c r="G42" s="1">
+        <v>20</v>
+      </c>
+      <c r="H42" s="1">
+        <v>20</v>
+      </c>
+      <c r="I42" s="1">
+        <v>5</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L42" s="1">
+        <v>100</v>
+      </c>
+      <c r="M42" s="2">
+        <v>1</v>
+      </c>
+      <c r="N42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O42" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A43" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" s="5">
+        <v>46111</v>
+      </c>
+      <c r="D43" s="1">
+        <v>5</v>
+      </c>
+      <c r="E43" s="1">
+        <v>20</v>
+      </c>
+      <c r="F43" s="1">
+        <v>30</v>
+      </c>
+      <c r="G43" s="1">
+        <v>20</v>
+      </c>
+      <c r="H43" s="1">
+        <v>20</v>
+      </c>
+      <c r="I43" s="1">
+        <v>5</v>
+      </c>
+      <c r="J43" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L43" s="1">
+        <v>100</v>
+      </c>
+      <c r="M43" s="2">
+        <v>1</v>
+      </c>
+      <c r="N43" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O43" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A44" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44" s="5">
+        <v>46129</v>
+      </c>
+      <c r="D44" s="1">
+        <v>5</v>
+      </c>
+      <c r="E44" s="1">
+        <v>20</v>
+      </c>
+      <c r="F44" s="1">
+        <v>30</v>
+      </c>
+      <c r="G44" s="1">
+        <v>15</v>
+      </c>
+      <c r="H44" s="1">
+        <v>20</v>
+      </c>
+      <c r="I44" s="1">
+        <v>5</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K44" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L44" s="1">
+        <v>95</v>
+      </c>
+      <c r="M44" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="N44" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O44" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A45" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" s="5">
+        <v>46108</v>
+      </c>
+      <c r="D45" s="1">
+        <v>5</v>
+      </c>
+      <c r="E45" s="1">
+        <v>20</v>
+      </c>
+      <c r="F45" s="1">
+        <v>30</v>
+      </c>
+      <c r="G45" s="1">
+        <v>20</v>
+      </c>
+      <c r="H45" s="1">
+        <v>10</v>
+      </c>
+      <c r="I45" s="1">
+        <v>5</v>
+      </c>
+      <c r="J45" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L45" s="1">
+        <v>90</v>
+      </c>
+      <c r="M45" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="N45" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O45" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" s="5">
+        <v>46126</v>
+      </c>
+      <c r="D46" s="1">
+        <v>5</v>
+      </c>
+      <c r="E46" s="1">
+        <v>20</v>
+      </c>
+      <c r="F46" s="1">
+        <v>30</v>
+      </c>
+      <c r="G46" s="1">
+        <v>20</v>
+      </c>
+      <c r="H46" s="1">
+        <v>20</v>
+      </c>
+      <c r="I46" s="1">
+        <v>5</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L46" s="1">
+        <v>100</v>
+      </c>
+      <c r="M46" s="2">
+        <v>1</v>
+      </c>
+      <c r="N46" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O46" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C47" s="5">
+        <v>46108</v>
+      </c>
+      <c r="D47" s="1">
+        <v>5</v>
+      </c>
+      <c r="E47" s="1">
+        <v>20</v>
+      </c>
+      <c r="F47" s="1">
+        <v>30</v>
+      </c>
+      <c r="G47" s="1">
+        <v>20</v>
+      </c>
+      <c r="H47" s="1">
+        <v>10</v>
+      </c>
+      <c r="I47" s="1">
+        <v>5</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L47" s="1">
+        <v>90</v>
+      </c>
+      <c r="M47" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="N47" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O47" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A48" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48" s="5">
+        <v>46111</v>
+      </c>
+      <c r="D48" s="1">
+        <v>5</v>
+      </c>
+      <c r="E48" s="1">
+        <v>20</v>
+      </c>
+      <c r="F48" s="1">
+        <v>30</v>
+      </c>
+      <c r="G48" s="1">
+        <v>20</v>
+      </c>
+      <c r="H48" s="1">
+        <v>20</v>
+      </c>
+      <c r="I48" s="1">
+        <v>5</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L48" s="1">
+        <v>100</v>
+      </c>
+      <c r="M48" s="2">
+        <v>1</v>
+      </c>
+      <c r="N48" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O48" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C49" s="5">
+        <v>46114</v>
+      </c>
+      <c r="D49" s="1">
+        <v>5</v>
+      </c>
+      <c r="E49" s="1">
+        <v>20</v>
+      </c>
+      <c r="F49" s="1">
+        <v>30</v>
+      </c>
+      <c r="G49" s="1">
+        <v>20</v>
+      </c>
+      <c r="H49" s="1">
+        <v>20</v>
+      </c>
+      <c r="I49" s="1">
+        <v>5</v>
+      </c>
+      <c r="J49" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K49" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L49" s="1">
+        <v>100</v>
+      </c>
+      <c r="M49" s="6">
+        <v>1</v>
+      </c>
+      <c r="N49" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O49" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A50" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C50" s="5">
+        <v>46129</v>
+      </c>
+      <c r="D50" s="1">
+        <v>5</v>
+      </c>
+      <c r="E50" s="1">
+        <v>20</v>
+      </c>
+      <c r="F50" s="1">
+        <v>30</v>
+      </c>
+      <c r="G50" s="1">
+        <v>20</v>
+      </c>
+      <c r="H50" s="1">
+        <v>20</v>
+      </c>
+      <c r="I50" s="1">
+        <v>5</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L50" s="1">
+        <v>100</v>
+      </c>
+      <c r="M50" s="6">
+        <v>1</v>
+      </c>
+      <c r="N50" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O50" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C51" s="5">
+        <v>46113</v>
+      </c>
+      <c r="D51" s="1">
+        <v>5</v>
+      </c>
+      <c r="E51" s="1">
+        <v>20</v>
+      </c>
+      <c r="F51" s="1">
+        <v>30</v>
+      </c>
+      <c r="G51" s="1">
+        <v>20</v>
+      </c>
+      <c r="H51" s="1">
+        <v>20</v>
+      </c>
+      <c r="I51" s="1">
+        <v>5</v>
+      </c>
+      <c r="J51" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L51" s="1">
+        <v>100</v>
+      </c>
+      <c r="M51" s="6">
+        <v>1</v>
+      </c>
+      <c r="N51" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O51" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A52" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C52" s="5">
+        <v>46118</v>
+      </c>
+      <c r="D52" s="1">
+        <v>5</v>
+      </c>
+      <c r="E52" s="1">
+        <v>20</v>
+      </c>
+      <c r="F52" s="1">
+        <v>30</v>
+      </c>
+      <c r="G52" s="1">
+        <v>20</v>
+      </c>
+      <c r="H52" s="1">
+        <v>0</v>
+      </c>
+      <c r="I52" s="1">
+        <v>5</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L52" s="1">
+        <v>80</v>
+      </c>
+      <c r="M52" s="6">
+        <v>0.8</v>
+      </c>
+      <c r="N52" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O52" s="1">
         <v>2026</v>
       </c>
     </row>
@@ -3015,16 +3720,16 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
update Grading raw file 05/11
</commit_message>
<xml_diff>
--- a/MAS_Call_Grading_Raw_Data.xlsx
+++ b/MAS_Call_Grading_Raw_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF6E91CA-7754-410E-96E4-7F4B9D1929F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{370AD02E-4819-4E2C-ABA1-ADBCE76976F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13610" yWindow="0" windowWidth="20840" windowHeight="13770" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="17970" windowHeight="13360" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="59">
   <si>
     <t>AssociateName</t>
   </si>
@@ -212,6 +212,9 @@
   <si>
     <t>Thomas.Gordon@lplfinancial.com</t>
   </si>
+  <si>
+    <t>May</t>
+  </si>
 </sst>
 </file>
 
@@ -325,8 +328,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O93" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:O93" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:O104" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:O104" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
   <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{F3FB1979-6840-4EDA-8F75-C44587A3E01A}" name="AssociateName"/>
     <tableColumn id="2" xr3:uid="{13759531-2D3E-4AB5-99AA-3CEAD45C9112}" name="ManagerTeam"/>
@@ -679,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E2710C-161E-4D4C-A0A9-FF139CE211A3}">
-  <dimension ref="A1:O93"/>
+  <dimension ref="A1:O104"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.54296875" customWidth="1"/>
@@ -4825,7 +4828,7 @@
       <c r="L88" s="1">
         <v>100</v>
       </c>
-      <c r="M88" s="6">
+      <c r="M88" s="2">
         <v>1</v>
       </c>
       <c r="N88" s="1" t="s">
@@ -4872,7 +4875,7 @@
       <c r="L89" s="1">
         <v>90</v>
       </c>
-      <c r="M89" s="6">
+      <c r="M89" s="2">
         <v>0.9</v>
       </c>
       <c r="N89" s="1" t="s">
@@ -4919,7 +4922,7 @@
       <c r="L90" s="1">
         <v>70</v>
       </c>
-      <c r="M90" s="6">
+      <c r="M90" s="2">
         <v>0.7</v>
       </c>
       <c r="N90" s="1" t="s">
@@ -4966,7 +4969,7 @@
       <c r="L91" s="1">
         <v>90</v>
       </c>
-      <c r="M91" s="6">
+      <c r="M91" s="2">
         <v>0.9</v>
       </c>
       <c r="N91" s="1" t="s">
@@ -5013,7 +5016,7 @@
       <c r="L92" s="1">
         <v>100</v>
       </c>
-      <c r="M92" s="6">
+      <c r="M92" s="2">
         <v>1</v>
       </c>
       <c r="N92" s="1" t="s">
@@ -5060,13 +5063,530 @@
       <c r="L93" s="1">
         <v>90</v>
       </c>
-      <c r="M93" s="6">
+      <c r="M93" s="2">
         <v>0.9</v>
       </c>
       <c r="N93" s="1" t="s">
         <v>28</v>
       </c>
       <c r="O93" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="94" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A94" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C94" s="5">
+        <v>46147</v>
+      </c>
+      <c r="D94" s="1">
+        <v>5</v>
+      </c>
+      <c r="E94" s="1">
+        <v>20</v>
+      </c>
+      <c r="F94" s="1">
+        <v>30</v>
+      </c>
+      <c r="G94" s="1">
+        <v>20</v>
+      </c>
+      <c r="H94" s="1">
+        <v>20</v>
+      </c>
+      <c r="I94" s="1">
+        <v>5</v>
+      </c>
+      <c r="J94" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K94" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L94" s="1">
+        <v>100</v>
+      </c>
+      <c r="M94" s="6">
+        <v>1</v>
+      </c>
+      <c r="N94" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O94" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="95" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A95" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C95" s="5">
+        <v>46148</v>
+      </c>
+      <c r="D95" s="1">
+        <v>5</v>
+      </c>
+      <c r="E95" s="1">
+        <v>20</v>
+      </c>
+      <c r="F95" s="1">
+        <v>30</v>
+      </c>
+      <c r="G95" s="1">
+        <v>20</v>
+      </c>
+      <c r="H95" s="1">
+        <v>20</v>
+      </c>
+      <c r="I95" s="1">
+        <v>5</v>
+      </c>
+      <c r="J95" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K95" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L95" s="1">
+        <v>100</v>
+      </c>
+      <c r="M95" s="6">
+        <v>1</v>
+      </c>
+      <c r="N95" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O95" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A96" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C96" s="5">
+        <v>46147</v>
+      </c>
+      <c r="D96" s="1">
+        <v>5</v>
+      </c>
+      <c r="E96" s="1">
+        <v>20</v>
+      </c>
+      <c r="F96" s="1">
+        <v>30</v>
+      </c>
+      <c r="G96" s="1">
+        <v>20</v>
+      </c>
+      <c r="H96" s="1">
+        <v>20</v>
+      </c>
+      <c r="I96" s="1">
+        <v>5</v>
+      </c>
+      <c r="J96" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K96" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L96" s="1">
+        <v>100</v>
+      </c>
+      <c r="M96" s="6">
+        <v>1</v>
+      </c>
+      <c r="N96" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O96" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A97" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C97" s="5">
+        <v>46149</v>
+      </c>
+      <c r="D97" s="1">
+        <v>5</v>
+      </c>
+      <c r="E97" s="1">
+        <v>20</v>
+      </c>
+      <c r="F97" s="1">
+        <v>30</v>
+      </c>
+      <c r="G97" s="1">
+        <v>20</v>
+      </c>
+      <c r="H97" s="1">
+        <v>20</v>
+      </c>
+      <c r="I97" s="1">
+        <v>5</v>
+      </c>
+      <c r="J97" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K97" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L97" s="1">
+        <v>100</v>
+      </c>
+      <c r="M97" s="6">
+        <v>1</v>
+      </c>
+      <c r="N97" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O97" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="98" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A98" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C98" s="5">
+        <v>46143</v>
+      </c>
+      <c r="D98" s="1">
+        <v>5</v>
+      </c>
+      <c r="E98" s="1">
+        <v>20</v>
+      </c>
+      <c r="F98" s="1">
+        <v>30</v>
+      </c>
+      <c r="G98" s="1">
+        <v>20</v>
+      </c>
+      <c r="H98" s="1">
+        <v>20</v>
+      </c>
+      <c r="I98" s="1">
+        <v>5</v>
+      </c>
+      <c r="J98" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K98" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L98" s="1">
+        <v>100</v>
+      </c>
+      <c r="M98" s="6">
+        <v>1</v>
+      </c>
+      <c r="N98" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O98" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A99" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C99" s="5">
+        <v>46148</v>
+      </c>
+      <c r="D99" s="1">
+        <v>5</v>
+      </c>
+      <c r="E99" s="1">
+        <v>20</v>
+      </c>
+      <c r="F99" s="1">
+        <v>30</v>
+      </c>
+      <c r="G99" s="1">
+        <v>20</v>
+      </c>
+      <c r="H99" s="1">
+        <v>20</v>
+      </c>
+      <c r="I99" s="1">
+        <v>5</v>
+      </c>
+      <c r="J99" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K99" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L99" s="1">
+        <v>100</v>
+      </c>
+      <c r="M99" s="6">
+        <v>1</v>
+      </c>
+      <c r="N99" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O99" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A100" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C100" s="5">
+        <v>46149</v>
+      </c>
+      <c r="D100" s="1">
+        <v>5</v>
+      </c>
+      <c r="E100" s="1">
+        <v>20</v>
+      </c>
+      <c r="F100" s="1">
+        <v>30</v>
+      </c>
+      <c r="G100" s="1">
+        <v>20</v>
+      </c>
+      <c r="H100" s="1">
+        <v>20</v>
+      </c>
+      <c r="I100" s="1">
+        <v>5</v>
+      </c>
+      <c r="J100" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K100" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L100" s="1">
+        <v>100</v>
+      </c>
+      <c r="M100" s="6">
+        <v>1</v>
+      </c>
+      <c r="N100" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O100" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A101" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C101" s="5">
+        <v>46149</v>
+      </c>
+      <c r="D101" s="1">
+        <v>5</v>
+      </c>
+      <c r="E101" s="1">
+        <v>20</v>
+      </c>
+      <c r="F101" s="1">
+        <v>30</v>
+      </c>
+      <c r="G101" s="1">
+        <v>20</v>
+      </c>
+      <c r="H101" s="1">
+        <v>20</v>
+      </c>
+      <c r="I101" s="1">
+        <v>5</v>
+      </c>
+      <c r="J101" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K101" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L101" s="1">
+        <v>100</v>
+      </c>
+      <c r="M101" s="6">
+        <v>1</v>
+      </c>
+      <c r="N101" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O101" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A102" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C102" s="5">
+        <v>46149</v>
+      </c>
+      <c r="D102" s="1">
+        <v>5</v>
+      </c>
+      <c r="E102" s="1">
+        <v>20</v>
+      </c>
+      <c r="F102" s="1">
+        <v>20</v>
+      </c>
+      <c r="G102" s="1">
+        <v>20</v>
+      </c>
+      <c r="H102" s="1">
+        <v>20</v>
+      </c>
+      <c r="I102" s="1">
+        <v>5</v>
+      </c>
+      <c r="J102" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K102" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L102" s="1">
+        <v>90</v>
+      </c>
+      <c r="M102" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="N102" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O102" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A103" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C103" s="5">
+        <v>46149</v>
+      </c>
+      <c r="D103" s="1">
+        <v>5</v>
+      </c>
+      <c r="E103" s="1">
+        <v>20</v>
+      </c>
+      <c r="F103" s="1">
+        <v>30</v>
+      </c>
+      <c r="G103" s="1">
+        <v>20</v>
+      </c>
+      <c r="H103" s="1">
+        <v>20</v>
+      </c>
+      <c r="I103" s="1">
+        <v>5</v>
+      </c>
+      <c r="J103" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K103" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L103" s="1">
+        <v>100</v>
+      </c>
+      <c r="M103" s="6">
+        <v>1</v>
+      </c>
+      <c r="N103" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O103" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A104" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C104" s="5">
+        <v>46148</v>
+      </c>
+      <c r="D104" s="1">
+        <v>5</v>
+      </c>
+      <c r="E104" s="1">
+        <v>20</v>
+      </c>
+      <c r="F104" s="1">
+        <v>30</v>
+      </c>
+      <c r="G104" s="1">
+        <v>20</v>
+      </c>
+      <c r="H104" s="1">
+        <v>20</v>
+      </c>
+      <c r="I104" s="1">
+        <v>5</v>
+      </c>
+      <c r="J104" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K104" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L104" s="1">
+        <v>100</v>
+      </c>
+      <c r="M104" s="6">
+        <v>1</v>
+      </c>
+      <c r="N104" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O104" s="1">
         <v>2026</v>
       </c>
     </row>
@@ -5372,28 +5892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
-    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B7CF5D77C2318A48AE3D01AED053E969" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7f98047a509e9e082d0d58dfbe71352c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c3d3890c-cedb-4996-8d69-32a58562dce0" xmlns:ns3="081083fe-e475-436e-8ac6-57ab24d1081c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="361f48e45990901628f9319c45e78890" ns2:_="" ns3:_="">
     <xsd:import namespace="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
@@ -5644,32 +6142,29 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
+    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AAD6C53-AA8B-4861-BD9E-3003633B2469}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E95F4425-7749-4603-B4BA-980799E13416}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5686,4 +6181,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AAD6C53-AA8B-4861-BD9E-3003633B2469}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updates charles grades 0608
</commit_message>
<xml_diff>
--- a/MAS_Call_Grading_Raw_Data.xlsx
+++ b/MAS_Call_Grading_Raw_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280F69CD-C803-4C98-A3D6-7276BF680D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76E3834-F7FC-416A-AEA2-04DAD0B03CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="790" yWindow="160" windowWidth="32080" windowHeight="13480" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
+    <workbookView xWindow="490" yWindow="230" windowWidth="30620" windowHeight="13480" xr2:uid="{57776DE4-8F31-45EC-A9ED-7D306CA54141}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Data" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="714" uniqueCount="53">
   <si>
     <t>AssociateName</t>
   </si>
@@ -310,8 +310,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:I120" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:I120" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}" name="tblRawData" displayName="tblRawData" ref="A1:I126" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:I126" xr:uid="{2EF4D820-248F-47FE-A171-6EE7F33C2BAC}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{F3FB1979-6840-4EDA-8F75-C44587A3E01A}" name="AssociateName"/>
     <tableColumn id="2" xr3:uid="{13759531-2D3E-4AB5-99AA-3CEAD45C9112}" name="ManagerTeam"/>
@@ -658,7 +658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02E2710C-161E-4D4C-A0A9-FF139CE211A3}">
-  <dimension ref="A1:I120"/>
+  <dimension ref="A1:I126"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
@@ -4025,7 +4025,7 @@
       <c r="F116" s="1">
         <v>100</v>
       </c>
-      <c r="G116" s="6">
+      <c r="G116" s="2">
         <v>1</v>
       </c>
       <c r="H116" s="1" t="s">
@@ -4054,7 +4054,7 @@
       <c r="F117" s="1">
         <v>90</v>
       </c>
-      <c r="G117" s="6">
+      <c r="G117" s="2">
         <v>0.9</v>
       </c>
       <c r="H117" s="1" t="s">
@@ -4083,7 +4083,7 @@
       <c r="F118" s="1">
         <v>100</v>
       </c>
-      <c r="G118" s="6">
+      <c r="G118" s="2">
         <v>1</v>
       </c>
       <c r="H118" s="1" t="s">
@@ -4112,7 +4112,7 @@
       <c r="F119" s="1">
         <v>100</v>
       </c>
-      <c r="G119" s="6">
+      <c r="G119" s="2">
         <v>1</v>
       </c>
       <c r="H119" s="1" t="s">
@@ -4141,13 +4141,187 @@
       <c r="F120" s="1">
         <v>100</v>
       </c>
-      <c r="G120" s="6">
+      <c r="G120" s="2">
         <v>1</v>
       </c>
       <c r="H120" s="1" t="s">
         <v>29</v>
       </c>
       <c r="I120" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A121" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C121" s="5">
+        <v>46178</v>
+      </c>
+      <c r="D121" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E121" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F121" s="1">
+        <v>100</v>
+      </c>
+      <c r="G121" s="6">
+        <v>1</v>
+      </c>
+      <c r="H121" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I121" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A122" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C122" s="5">
+        <v>46178</v>
+      </c>
+      <c r="D122" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F122" s="1">
+        <v>100</v>
+      </c>
+      <c r="G122" s="6">
+        <v>1</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I122" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A123" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C123" s="5">
+        <v>46178</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F123" s="1">
+        <v>90</v>
+      </c>
+      <c r="G123" s="6">
+        <v>0.9</v>
+      </c>
+      <c r="H123" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I123" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A124" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C124" s="5">
+        <v>46177</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E124" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F124" s="1">
+        <v>100</v>
+      </c>
+      <c r="G124" s="6">
+        <v>1</v>
+      </c>
+      <c r="H124" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I124" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A125" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C125" s="5">
+        <v>46178</v>
+      </c>
+      <c r="D125" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F125" s="1">
+        <v>95</v>
+      </c>
+      <c r="G125" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="H125" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I125" s="1">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A126" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C126" s="5">
+        <v>46178</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E126" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F126" s="1">
+        <v>100</v>
+      </c>
+      <c r="G126" s="6">
+        <v>1</v>
+      </c>
+      <c r="H126" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I126" s="1">
         <v>2026</v>
       </c>
     </row>
@@ -4453,28 +4627,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
-    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B7CF5D77C2318A48AE3D01AED053E969" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7f98047a509e9e082d0d58dfbe71352c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c3d3890c-cedb-4996-8d69-32a58562dce0" xmlns:ns3="081083fe-e475-436e-8ac6-57ab24d1081c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="361f48e45990901628f9319c45e78890" ns2:_="" ns3:_="">
     <xsd:import namespace="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
@@ -4725,32 +4877,29 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AAD6C53-AA8B-4861-BD9E-3003633B2469}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
+    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E95F4425-7749-4603-B4BA-980799E13416}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4767,4 +4916,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AAD6C53-AA8B-4861-BD9E-3003633B2469}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810E8512-413E-4D31-94ED-3194BEC41610}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>